<commit_message>
eerste aanpassingen naar de WADAR test
nog niet perfect, maar getest met de eerste WADAR uitdraai
</commit_message>
<xml_diff>
--- a/mappings/locations-raw.xlsx
+++ b/mappings/locations-raw.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>LOCOMS</t>
+          <t>locatie_code</t>
         </is>
       </c>
     </row>
@@ -459,79 +459,79 @@
       <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Hansweert geul</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NL89_SASVGT</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Sas van Gent</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NL89_SASVGT</t>
+          <t>NL89_SCHAARVODDL</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Sas van Gent</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Sas van Gent</t>
-        </is>
-      </c>
+          <t>Schaar van Ouden Doel</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NL89_SCHAARVODDL</t>
+          <t>NL_TERNZBI20</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Schaar van Ouden Doel</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Schaar van Ouden Doel</t>
-        </is>
-      </c>
+          <t>Terneuzen</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NL_TERNZBI20</t>
+          <t>NL89_VLISSGBISSVH</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Terneuzen</t>
+          <t>Vlissingen</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Terneuzen boei 20</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NL95_WALCRN2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Walcheren 2</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NL89_VLISSGBISSVH</t>
+          <t>NL89_WISSKKE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Vlissingen</t>
+          <t>Wissenkerke</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -541,46 +541,61 @@
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Vlissingen boei SSVH</t>
+          <t>hansweert.geul</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>NL95_WALCRN2</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Walcheren 2</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>sasvangent.grens</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Walcheren 2 km uit de kust</t>
+          <t>schaarvanoudendoel</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>NL89_WISSKKE</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Wissenkerke</t>
-        </is>
-      </c>
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Wissenkerke</t>
+          <t>terneuzen.boei20</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>vlissingen.boeissvh</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>walcheren.2kmuitdekust</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>wissenkerke</t>
         </is>
       </c>
     </row>

</xml_diff>